<commit_message>
feat: rename XON CARGO, normalize types and fix Umumiy hisobot Excel formulas for custom types
</commit_message>
<xml_diff>
--- a/assets/umumiy_hisobot_shabloni.xlsx
+++ b/assets/umumiy_hisobot_shabloni.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="14020" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Лист1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Лист1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -678,7 +678,7 @@
     <row r="11">
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>one</t>
+          <t>oneway</t>
         </is>
       </c>
       <c r="C11" s="5" t="n">

</xml_diff>